<commit_message>
CSV File export run
</commit_message>
<xml_diff>
--- a/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
+++ b/InputData/bldgs/BPSfDSPC/BAU Perc Subsidy for Distributed Solar PV Capacity.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27720"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Richa.richa\Downloads\BPSfDSPC\BPSfDSPC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\India EPS\InputData\bldgs\BPSfDSPC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{C4CD6C72-4998-4F43-948F-FC077E0F061A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E19FBF4E-07E7-4597-84B9-E1CCC548F6AD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F82666B1-E486-4231-844E-CFB01D9499C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="7" r:id="rId1"/>
-    <sheet name="BPSfDSPV" sheetId="8" r:id="rId2"/>
+    <sheet name="BPSfDSPC" sheetId="8" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -82,7 +82,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -434,24 +434,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="61.5703125" customWidth="1"/>
     <col min="5" max="5" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -459,10 +460,10 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -475,17 +476,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <sheetPr>
+  <sheetPr codeName="Sheet2">
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AZ7"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52">
+    <row r="1" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>5</v>
       </c>
@@ -640,7 +641,7 @@
         <v>2070</v>
       </c>
     </row>
-    <row r="2" spans="1:52">
+    <row r="2" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -796,7 +797,7 @@
       </c>
       <c r="AZ2" s="5"/>
     </row>
-    <row r="3" spans="1:52">
+    <row r="3" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -952,7 +953,7 @@
       </c>
       <c r="AZ3" s="5"/>
     </row>
-    <row r="4" spans="1:52">
+    <row r="4" spans="1:52" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1108,13 +1109,13 @@
       </c>
       <c r="AZ4" s="5"/>
     </row>
-    <row r="5" spans="1:52">
+    <row r="5" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
     </row>
-    <row r="6" spans="1:52">
+    <row r="6" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
     </row>
-    <row r="7" spans="1:52">
+    <row r="7" spans="1:52" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
     </row>
   </sheetData>
@@ -1124,6 +1125,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A251C7805F896F47A4F48569C73A0799" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="77cd1fc208aa16a525090c2a27f33c66">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f3083de3-5d4e-49f2-a3cd-0aeb079e6739" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d77402130d0e9b5bbfbb66ed18db98d9" ns2:_="">
     <xsd:import namespace="f3083de3-5d4e-49f2-a3cd-0aeb079e6739"/>
@@ -1267,12 +1274,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1283,13 +1284,36 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C255835-D2CA-4403-8823-9819BA3F6B81}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3314045-B15D-4491-8336-AA71AEA28892}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3314045-B15D-4491-8336-AA71AEA28892}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4C255835-D2CA-4403-8823-9819BA3F6B81}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f3083de3-5d4e-49f2-a3cd-0aeb079e6739"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27410CAB-AF69-4BF0-9B1A-348171EF6757}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27410CAB-AF69-4BF0-9B1A-348171EF6757}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>